<commit_message>
Added new Result Limits
</commit_message>
<xml_diff>
--- a/scripts/modify_LIS_scripts/Laborwerte_zum_behalten_mit_Normwerten.xlsx
+++ b/scripts/modify_LIS_scripts/Laborwerte_zum_behalten_mit_Normwerten.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Workspace\Bahmni_Project\KIS-Projekt\scripts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Workspace\Bahmni_Project\KIS-Projekt\scripts\modify_LIS_scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{458A1DE0-468C-4927-B5E6-4814904F0B11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{866633BE-A866-4E45-BA53-46BA82D2B0AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="7155" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="333">
   <si>
     <t>Name</t>
   </si>
@@ -1011,13 +1011,37 @@
   </si>
   <si>
     <t>f = female, m= male</t>
+  </si>
+  <si>
+    <t>Glomerular filtration rate, calculated</t>
+  </si>
+  <si>
+    <t>GFR nach CKD-EPI</t>
+  </si>
+  <si>
+    <t>161133AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+  </si>
+  <si>
+    <t>N-terminal pro brain natriuretic peptide (NT-proBNP) measurement</t>
+  </si>
+  <si>
+    <t>NT-pro-BNP</t>
+  </si>
+  <si>
+    <t>166017AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+  </si>
+  <si>
+    <t>ml/min</t>
+  </si>
+  <si>
+    <t>ng/l</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1390,8 +1414,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X104"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <dimension ref="A1:X106"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="67.28515625" customWidth="1"/>
     <col min="2" max="2" width="44.140625" customWidth="1"/>
@@ -1419,7 +1443,7 @@
     <col min="24" max="24" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1493,7 +1517,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:24">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -1513,7 +1537,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:24">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -1530,7 +1554,7 @@
         <v>7.45</v>
       </c>
     </row>
-    <row r="4" spans="1:24">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>31</v>
       </c>
@@ -1550,7 +1574,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:24">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>35</v>
       </c>
@@ -1570,7 +1594,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:24">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>38</v>
       </c>
@@ -1590,7 +1614,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:24">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>41</v>
       </c>
@@ -1622,7 +1646,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:24">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>47</v>
       </c>
@@ -1642,7 +1666,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="9" spans="1:24">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="3" t="s">
         <v>51</v>
@@ -1661,7 +1685,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:24">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>54</v>
       </c>
@@ -1681,7 +1705,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:24">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>57</v>
       </c>
@@ -1701,7 +1725,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:24">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>60</v>
       </c>
@@ -1721,7 +1745,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:24">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>63</v>
       </c>
@@ -1741,7 +1765,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:24">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>66</v>
       </c>
@@ -1761,7 +1785,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:24">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>69</v>
       </c>
@@ -1781,7 +1805,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:24">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>72</v>
       </c>
@@ -1801,7 +1825,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>76</v>
       </c>
@@ -1833,7 +1857,7 @@
         <v>5.9</v>
       </c>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>80</v>
       </c>
@@ -1853,7 +1877,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:14">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>83</v>
       </c>
@@ -1873,7 +1897,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:14">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>87</v>
       </c>
@@ -1893,7 +1917,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>91</v>
       </c>
@@ -1913,7 +1937,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="22" spans="1:14">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>95</v>
       </c>
@@ -1945,7 +1969,7 @@
         <v>17.2</v>
       </c>
     </row>
-    <row r="23" spans="1:14">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>99</v>
       </c>
@@ -1965,7 +1989,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:14">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>102</v>
       </c>
@@ -1994,7 +2018,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="25" spans="1:14">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>105</v>
       </c>
@@ -2014,7 +2038,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="26" spans="1:14">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>108</v>
       </c>
@@ -2034,7 +2058,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="27" spans="1:14">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>112</v>
       </c>
@@ -2054,7 +2078,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="28" spans="1:14">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>115</v>
       </c>
@@ -2074,7 +2098,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="29" spans="1:14">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>118</v>
       </c>
@@ -2094,7 +2118,7 @@
         <v>0.39</v>
       </c>
     </row>
-    <row r="30" spans="1:14">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>121</v>
       </c>
@@ -2114,7 +2138,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="31" spans="1:14">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>125</v>
       </c>
@@ -2146,7 +2170,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="32" spans="1:14">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>129</v>
       </c>
@@ -2166,7 +2190,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="33" spans="1:24">
+    <row r="33" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>132</v>
       </c>
@@ -2186,7 +2210,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="34" spans="1:24">
+    <row r="34" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>135</v>
       </c>
@@ -2206,7 +2230,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="35" spans="1:24">
+    <row r="35" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>139</v>
       </c>
@@ -2238,7 +2262,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="36" spans="1:24">
+    <row r="36" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>142</v>
       </c>
@@ -2258,7 +2282,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="37" spans="1:24">
+    <row r="37" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>146</v>
       </c>
@@ -2278,7 +2302,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="38" spans="1:24">
+    <row r="38" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>149</v>
       </c>
@@ -2298,7 +2322,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:24">
+    <row r="39" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>153</v>
       </c>
@@ -2318,7 +2342,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="40" spans="1:24">
+    <row r="40" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>156</v>
       </c>
@@ -2338,7 +2362,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="41" spans="1:24">
+    <row r="41" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>159</v>
       </c>
@@ -2358,7 +2382,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="42" spans="1:24">
+    <row r="42" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>162</v>
       </c>
@@ -2378,7 +2402,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="43" spans="1:24">
+    <row r="43" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>165</v>
       </c>
@@ -2398,7 +2422,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:24">
+    <row r="44" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A44" s="3"/>
       <c r="B44" s="3" t="s">
         <v>168</v>
@@ -2426,7 +2450,7 @@
         <v>12.9</v>
       </c>
     </row>
-    <row r="45" spans="1:24">
+    <row r="45" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>171</v>
       </c>
@@ -2446,7 +2470,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="46" spans="1:24">
+    <row r="46" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>175</v>
       </c>
@@ -2520,7 +2544,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="47" spans="1:24">
+    <row r="47" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>178</v>
       </c>
@@ -2540,7 +2564,7 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="48" spans="1:24">
+    <row r="48" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A48" s="3"/>
       <c r="B48" s="3" t="s">
         <v>181</v>
@@ -2559,7 +2583,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="49" spans="1:14">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>183</v>
       </c>
@@ -2591,7 +2615,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="50" spans="1:14">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>186</v>
       </c>
@@ -2623,7 +2647,7 @@
         <v>8.1999999999999993</v>
       </c>
     </row>
-    <row r="51" spans="1:14">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>189</v>
       </c>
@@ -2661,7 +2685,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="52" spans="1:14">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>192</v>
       </c>
@@ -2699,7 +2723,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="53" spans="1:14">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="3"/>
       <c r="B53" s="3" t="s">
         <v>195</v>
@@ -2718,7 +2742,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="54" spans="1:14">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>197</v>
       </c>
@@ -2738,7 +2762,7 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="55" spans="1:14">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="3"/>
       <c r="B55" s="3" t="s">
         <v>200</v>
@@ -2757,7 +2781,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:14">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>203</v>
       </c>
@@ -2777,7 +2801,7 @@
         <v>2.65</v>
       </c>
     </row>
-    <row r="57" spans="1:14">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>206</v>
       </c>
@@ -2797,7 +2821,7 @@
         <v>1.35</v>
       </c>
     </row>
-    <row r="58" spans="1:14">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>209</v>
       </c>
@@ -2817,7 +2841,7 @@
         <v>1.35</v>
       </c>
     </row>
-    <row r="59" spans="1:14">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>212</v>
       </c>
@@ -2837,7 +2861,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="60" spans="1:14">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>215</v>
       </c>
@@ -2869,7 +2893,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="61" spans="1:14">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>218</v>
       </c>
@@ -2901,7 +2925,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="62" spans="1:14">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>221</v>
       </c>
@@ -2933,7 +2957,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="63" spans="1:14">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>224</v>
       </c>
@@ -2953,7 +2977,7 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="64" spans="1:14">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>227</v>
       </c>
@@ -2973,7 +2997,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="65" spans="1:14">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>230</v>
       </c>
@@ -2993,7 +3017,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="66" spans="1:14">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>233</v>
       </c>
@@ -3025,7 +3049,7 @@
         <v>1.06</v>
       </c>
     </row>
-    <row r="67" spans="1:14">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>236</v>
       </c>
@@ -3045,7 +3069,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="68" spans="1:14">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>239</v>
       </c>
@@ -3065,7 +3089,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="69" spans="1:14">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>243</v>
       </c>
@@ -3085,7 +3109,7 @@
         <v>1.45</v>
       </c>
     </row>
-    <row r="70" spans="1:14">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>246</v>
       </c>
@@ -3117,7 +3141,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="71" spans="1:14">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>249</v>
       </c>
@@ -3137,7 +3161,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="72" spans="1:14">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>252</v>
       </c>
@@ -3157,7 +3181,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="73" spans="1:14">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>256</v>
       </c>
@@ -3177,7 +3201,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="74" spans="1:14">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A74" s="3"/>
       <c r="B74" s="3" t="s">
         <v>259</v>
@@ -3196,7 +3220,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="75" spans="1:14">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A75" s="3"/>
       <c r="B75" s="3" t="s">
         <v>261</v>
@@ -3215,7 +3239,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="76" spans="1:14">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>263</v>
       </c>
@@ -3235,7 +3259,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="77" spans="1:14">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>266</v>
       </c>
@@ -3255,7 +3279,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="78" spans="1:14">
+    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A78" s="3"/>
       <c r="B78" s="3" t="s">
         <v>269</v>
@@ -3274,7 +3298,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="79" spans="1:14">
+    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>272</v>
       </c>
@@ -3294,7 +3318,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="80" spans="1:14">
+    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>275</v>
       </c>
@@ -3314,7 +3338,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="81" spans="1:14">
+    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A81" s="3"/>
       <c r="B81" s="3" t="s">
         <v>278</v>
@@ -3333,7 +3357,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="82" spans="1:14">
+    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A82" s="3"/>
       <c r="B82" s="3" t="s">
         <v>280</v>
@@ -3352,7 +3376,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="83" spans="1:14">
+    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>282</v>
       </c>
@@ -3372,7 +3396,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="84" spans="1:14">
+    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>286</v>
       </c>
@@ -3404,91 +3428,91 @@
         <v>40</v>
       </c>
     </row>
-    <row r="87" spans="1:14">
-      <c r="A87" s="2" t="s">
+    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>325</v>
+      </c>
+      <c r="B85" t="s">
+        <v>326</v>
+      </c>
+      <c r="C85" t="s">
+        <v>327</v>
+      </c>
+      <c r="D85" t="s">
+        <v>331</v>
+      </c>
+      <c r="H85">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>328</v>
+      </c>
+      <c r="B86" t="s">
+        <v>329</v>
+      </c>
+      <c r="C86" t="s">
+        <v>330</v>
+      </c>
+      <c r="D86" t="s">
+        <v>332</v>
+      </c>
+      <c r="I86">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="89" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A89" s="2" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="88" spans="1:14">
-      <c r="A88" t="s">
+    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
         <v>290</v>
       </c>
-      <c r="B88" s="4" t="s">
+      <c r="B90" s="4" t="s">
         <v>291</v>
       </c>
-      <c r="C88" t="s">
+      <c r="C90" t="s">
         <v>292</v>
       </c>
-      <c r="D88" t="s">
+      <c r="D90" t="s">
         <v>94</v>
       </c>
-      <c r="H88">
+      <c r="H90">
         <v>1015</v>
       </c>
-      <c r="I88">
+      <c r="I90">
         <v>1030</v>
       </c>
     </row>
-    <row r="89" spans="1:14">
-      <c r="A89" t="s">
+    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
         <v>293</v>
       </c>
-      <c r="B89" s="4" t="s">
+      <c r="B91" s="4" t="s">
         <v>294</v>
       </c>
-      <c r="C89" t="s">
+      <c r="C91" t="s">
         <v>295</v>
       </c>
-      <c r="H89">
+      <c r="H91">
         <v>4.8</v>
       </c>
-      <c r="I89">
+      <c r="I91">
         <v>7.6</v>
       </c>
     </row>
-    <row r="90" spans="1:14">
-      <c r="A90" t="s">
+    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
         <v>296</v>
       </c>
-      <c r="B90" s="4" t="s">
+      <c r="B92" s="4" t="s">
         <v>297</v>
       </c>
-      <c r="C90" t="s">
+      <c r="C92" t="s">
         <v>298</v>
-      </c>
-      <c r="D90" s="6"/>
-      <c r="E90" s="6"/>
-      <c r="F90" s="6"/>
-      <c r="G90" s="6"/>
-      <c r="H90" s="6"/>
-      <c r="I90" s="6"/>
-    </row>
-    <row r="91" spans="1:14">
-      <c r="A91" t="s">
-        <v>299</v>
-      </c>
-      <c r="B91" s="4" t="s">
-        <v>300</v>
-      </c>
-      <c r="C91" t="s">
-        <v>301</v>
-      </c>
-      <c r="D91" s="6"/>
-      <c r="E91" s="6"/>
-      <c r="F91" s="6"/>
-      <c r="G91" s="6"/>
-      <c r="H91" s="6"/>
-      <c r="I91" s="6"/>
-    </row>
-    <row r="92" spans="1:14">
-      <c r="A92" t="s">
-        <v>302</v>
-      </c>
-      <c r="B92" s="4" t="s">
-        <v>303</v>
-      </c>
-      <c r="C92" t="s">
-        <v>304</v>
       </c>
       <c r="D92" s="6"/>
       <c r="E92" s="6"/>
@@ -3497,15 +3521,15 @@
       <c r="H92" s="6"/>
       <c r="I92" s="6"/>
     </row>
-    <row r="93" spans="1:14">
+    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="C93" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="D93" s="6"/>
       <c r="E93" s="6"/>
@@ -3514,15 +3538,15 @@
       <c r="H93" s="6"/>
       <c r="I93" s="6"/>
     </row>
-    <row r="94" spans="1:14">
+    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="C94" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="D94" s="6"/>
       <c r="E94" s="6"/>
@@ -3531,15 +3555,15 @@
       <c r="H94" s="6"/>
       <c r="I94" s="6"/>
     </row>
-    <row r="95" spans="1:14">
+    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="C95" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="D95" s="6"/>
       <c r="E95" s="6"/>
@@ -3548,67 +3572,101 @@
       <c r="H95" s="6"/>
       <c r="I95" s="6"/>
     </row>
-    <row r="96" spans="1:14">
-      <c r="B96" s="4"/>
-    </row>
-    <row r="97" spans="1:9">
-      <c r="A97" s="2" t="s">
+    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>308</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="C96" t="s">
+        <v>310</v>
+      </c>
+      <c r="D96" s="6"/>
+      <c r="E96" s="6"/>
+      <c r="F96" s="6"/>
+      <c r="G96" s="6"/>
+      <c r="H96" s="6"/>
+      <c r="I96" s="6"/>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>311</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="C97" t="s">
+        <v>313</v>
+      </c>
+      <c r="D97" s="6"/>
+      <c r="E97" s="6"/>
+      <c r="F97" s="6"/>
+      <c r="G97" s="6"/>
+      <c r="H97" s="6"/>
+      <c r="I97" s="6"/>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B98" s="4"/>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A99" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="B97" s="4"/>
-    </row>
-    <row r="98" spans="1:9">
-      <c r="A98" t="s">
+      <c r="B99" s="4"/>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
         <v>315</v>
       </c>
-      <c r="B98" s="4" t="s">
+      <c r="B100" s="4" t="s">
         <v>316</v>
       </c>
-      <c r="C98" t="s">
+      <c r="C100" t="s">
         <v>317</v>
       </c>
-      <c r="D98" t="s">
+      <c r="D100" t="s">
         <v>318</v>
       </c>
-      <c r="H98">
-        <v>0</v>
-      </c>
-      <c r="I98">
+      <c r="H100">
+        <v>0</v>
+      </c>
+      <c r="I100">
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:9">
-      <c r="A99" t="s">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
         <v>319</v>
       </c>
-      <c r="B99" s="4" t="s">
+      <c r="B101" s="4" t="s">
         <v>320</v>
       </c>
-      <c r="C99" t="s">
+      <c r="C101" t="s">
         <v>321</v>
       </c>
-      <c r="D99" t="s">
+      <c r="D101" t="s">
         <v>318</v>
       </c>
-      <c r="H99">
-        <v>0</v>
-      </c>
-      <c r="I99">
+      <c r="H101">
+        <v>0</v>
+      </c>
+      <c r="I101">
         <v>4</v>
       </c>
     </row>
-    <row r="102" spans="1:9">
-      <c r="A102" s="3" t="s">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A104" s="3" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="103" spans="1:9">
-      <c r="A103" s="6" t="s">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A105" s="6" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="104" spans="1:9">
-      <c r="A104" t="s">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
         <v>324</v>
       </c>
     </row>

</xml_diff>